<commit_message>
Update tobacco company in AddictO_Organisation_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Organisation_Defs.xlsx
+++ b/inputs/AddictO_Organisation_Defs.xlsx
@@ -463,97 +463,97 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Synonyms</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-ontology</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Why fuzzy</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has role'</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has part'</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Cross reference</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Curator note</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Informal definition</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>E-CigO</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>To be reviewed by</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Examples of usage</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Definition source</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-ontology</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>BFO entity</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has role'</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has part'</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Curator note</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Cross reference</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Synonyms</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Fuzzy set</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Examples of usage</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>E-CigO</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Why fuzzy</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>To be reviewed by</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -580,14 +580,10 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>A commercial organisation that deals with nicotine products or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
           <t>commercial organisation</t>
         </is>
       </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="inlineStr">
@@ -595,32 +591,36 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n">
-        <v>0</v>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>A commercial organisation that deals with nicotine products or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V2" s="2" t="n"/>
+      <c r="V2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="W2" s="2" t="n"/>
     </row>
     <row r="3">
@@ -639,10 +639,14 @@
           <t>A charity that provides funding for research, prevention, treatment or care relating to alcohol use.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>organisation</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>organisation</t>
+          <t xml:space="preserve">alcohol harm prevention organisation </t>
         </is>
       </c>
       <c r="F3" s="3" t="n"/>
@@ -652,20 +656,12 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">alcohol harm prevention organisation </t>
-        </is>
-      </c>
+      <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -673,15 +669,15 @@
       </c>
       <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="n"/>
+      <c r="R3" s="3" t="n"/>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -689,7 +685,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V3" s="3" t="n"/>
+      <c r="V3" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W3" s="3" t="n"/>
     </row>
     <row r="4">
@@ -708,12 +708,12 @@
           <t>An industry that is realised in the manufacture and sale of alcoholic beverages.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
+      <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="inlineStr">
@@ -721,11 +721,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
+      <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n"/>
@@ -738,15 +734,15 @@
       </c>
       <c r="P4" s="4" t="n"/>
       <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S4" s="4" t="n"/>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>realizable entity</t>
         </is>
       </c>
       <c r="U4" s="4" t="inlineStr">
@@ -754,7 +750,11 @@
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V4" s="4" t="n"/>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W4" s="4" t="n"/>
     </row>
     <row r="5">
@@ -773,12 +773,12 @@
           <t>An organisation that undertakes assays for presence or amounts of chemicals in specimens</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="inlineStr">
@@ -786,11 +786,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Role </t>
-        </is>
-      </c>
+      <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>
@@ -803,15 +799,15 @@
       </c>
       <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S5" s="3" t="n"/>
+      <c r="R5" s="3" t="n"/>
+      <c r="S5" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t xml:space="preserve">Role </t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -819,7 +815,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V5" s="3" t="n"/>
+      <c r="V5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W5" s="3" t="n"/>
     </row>
     <row r="6">
@@ -838,10 +838,14 @@
           <t>A charity that provides funding for cancer-related research, prevention, treatment or care.</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">organisation </t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">organisation </t>
+          <t xml:space="preserve">cancer prevention organisation </t>
         </is>
       </c>
       <c r="F6" s="3" t="n"/>
@@ -851,34 +855,26 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Role </t>
-        </is>
-      </c>
+      <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cancer prevention organisation </t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" s="3" t="n"/>
+      <c r="R6" s="3" t="n"/>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t xml:space="preserve">Role </t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -886,7 +882,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V6" s="3" t="n"/>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W6" s="3" t="n"/>
     </row>
     <row r="7">
@@ -905,12 +905,12 @@
           <t xml:space="preserve">An organisation that is engaged in the growth, manufacture, preparation for sale, shipment, advertisement, or distribution of cannabis products. </t>
         </is>
       </c>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="inlineStr">
@@ -918,11 +918,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Role </t>
-        </is>
-      </c>
+      <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
@@ -935,15 +931,15 @@
       </c>
       <c r="P7" s="3" t="n"/>
       <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S7" s="3" t="n"/>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH; KS</t>
+        </is>
+      </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>SC; JH; KS</t>
+          <t xml:space="preserve">Role </t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -951,7 +947,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V7" s="3" t="n"/>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W7" s="3" t="n"/>
     </row>
     <row r="8">
@@ -970,12 +970,12 @@
           <t>An industry that is realised in the manufacture and sale of cannabis.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
+      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="inlineStr">
@@ -983,11 +983,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
+      <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
@@ -1000,15 +996,15 @@
       </c>
       <c r="P8" s="2" t="n"/>
       <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="n"/>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>realizable entity</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
@@ -1016,7 +1012,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V8" s="2" t="n"/>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W8" s="2" t="n"/>
     </row>
     <row r="9">
@@ -1035,12 +1035,12 @@
           <t xml:space="preserve">A cannabis retailer that has a physical outlet. </t>
         </is>
       </c>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>cannabis retailer</t>
         </is>
       </c>
+      <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="inlineStr">
@@ -1048,11 +1048,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Role </t>
-        </is>
-      </c>
+      <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
@@ -1065,15 +1061,15 @@
       </c>
       <c r="P9" s="3" t="n"/>
       <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S9" s="3" t="n"/>
+      <c r="R9" s="3" t="n"/>
+      <c r="S9" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t xml:space="preserve">Role </t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
@@ -1081,7 +1077,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V9" s="3" t="n"/>
+      <c r="V9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W9" s="3" t="n"/>
     </row>
     <row r="10">
@@ -1100,12 +1100,12 @@
           <t xml:space="preserve">A cannabis company that predominantly sells cannabis products and related merchandise. </t>
         </is>
       </c>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">cannabis company </t>
         </is>
       </c>
+      <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="inlineStr">
@@ -1113,11 +1113,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Role </t>
-        </is>
-      </c>
+      <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="n"/>
@@ -1130,15 +1126,15 @@
       </c>
       <c r="P10" s="3" t="n"/>
       <c r="Q10" s="3" t="n"/>
-      <c r="R10" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S10" s="3" t="n"/>
+      <c r="R10" s="3" t="n"/>
+      <c r="S10" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t xml:space="preserve">Role </t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -1146,7 +1142,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V10" s="3" t="n"/>
+      <c r="V10" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W10" s="3" t="n"/>
     </row>
     <row r="11">
@@ -1165,12 +1165,12 @@
           <t xml:space="preserve">An organisation that raises and distributes funds for charitable purposes. </t>
         </is>
       </c>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="inlineStr">
@@ -1178,30 +1178,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="n"/>
+      <c r="O11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>RW; CN</t>
+        </is>
+      </c>
       <c r="Q11" s="2" t="n"/>
-      <c r="R11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S11" s="2" t="n"/>
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U11" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="V11" s="2" t="inlineStr">
         <is>
-          <t>RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W11" s="2" t="n"/>
@@ -1234,14 +1234,10 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>An organisation whose main goal is making money by selling products or services.</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="inlineStr">
@@ -1249,32 +1245,36 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
-      <c r="O12" s="2" t="n">
-        <v>0</v>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>An organisation whose main goal is making money by selling products or services.</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="P12" s="2" t="n"/>
       <c r="Q12" s="2" t="n"/>
-      <c r="R12" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="n"/>
-      <c r="T12" s="2" t="n"/>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V12" s="2" t="n"/>
+      <c r="V12" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="W12" s="2" t="n"/>
     </row>
     <row r="13">
@@ -1295,14 +1295,10 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>A commercial organisation that deals with e-cigarettes or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
           <t>commercial organisation</t>
         </is>
       </c>
+      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="n"/>
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="inlineStr">
@@ -1310,32 +1306,36 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
-      <c r="O13" s="2" t="n">
-        <v>0</v>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>A commercial organisation that deals with e-cigarettes or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="P13" s="2" t="n"/>
       <c r="Q13" s="2" t="n"/>
-      <c r="R13" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="R13" s="2" t="n"/>
       <c r="S13" s="2" t="n"/>
-      <c r="T13" s="2" t="n"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V13" s="2" t="n"/>
+      <c r="V13" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" s="2" t="n"/>
     </row>
     <row r="14">
@@ -1354,10 +1354,14 @@
           <t>An industry that is realised in the manufacture and sale of e-cigarettes, e-cigarette components and e-liquid.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>industry</t>
+        </is>
+      </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>industry</t>
+          <t>E-Cig industry</t>
         </is>
       </c>
       <c r="F14" s="4" t="n"/>
@@ -1367,38 +1371,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
+      <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
       <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">I have added here promotion of - this sets industry apart from manufactureres of but also includes these types of company. </t>
         </is>
       </c>
-      <c r="M14" s="4" t="n"/>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>E-Cig industry</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="N14" s="4" t="n"/>
+      <c r="O14" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="n"/>
-      <c r="R14" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S14" s="4" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>realizable entity</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
@@ -1406,7 +1402,11 @@
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V14" s="4" t="n"/>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W14" s="4" t="n"/>
     </row>
     <row r="15">
@@ -1425,10 +1425,14 @@
           <t>A e-cigarette company that predominantly sells e-cigarettes, e-cigarette components or e-liquid to consumers.</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>e-cigarette company</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>e-cigarette company</t>
+          <t>E-Cig shop; E-cig Industry; E-Cig merchant; vape shop; vape retailer</t>
         </is>
       </c>
       <c r="F15" s="3" t="n"/>
@@ -1438,34 +1442,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
+      <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="inlineStr">
-        <is>
-          <t>E-Cig shop; E-cig Industry; E-Cig merchant; vape shop; vape retailer</t>
-        </is>
-      </c>
-      <c r="O15" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P15" s="3" t="n"/>
+      <c r="N15" s="3" t="n"/>
+      <c r="O15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q15" s="3" t="n"/>
-      <c r="R15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" s="3" t="n"/>
+      <c r="R15" s="3" t="n"/>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH</t>
+        </is>
+      </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>SC; JH</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="U15" s="3" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="V15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W15" s="3" t="n"/>
@@ -1496,12 +1496,12 @@
           <t>An e-cigarette shop is an e-cigarette retailer that has a physical outlet.</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>e-cigarette retailer</t>
         </is>
       </c>
+      <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="inlineStr">
@@ -1509,30 +1509,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
+      <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="n"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n"/>
       <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P16" s="3" t="n"/>
+      <c r="O16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q16" s="3" t="n"/>
-      <c r="R16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S16" s="3" t="n"/>
+      <c r="R16" s="3" t="n"/>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH</t>
+        </is>
+      </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>SC; JH</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="U16" s="3" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="V16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W16" s="3" t="n"/>
@@ -1563,12 +1563,12 @@
           <t>An e-cigarette organisation that is engaged in the growth, manufacture, preparation for sale, shipment, advertisement, or distribution of e-liquid.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>e-cigarette organisation</t>
         </is>
       </c>
+      <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="inlineStr">
@@ -1576,30 +1576,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
+      <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
       <c r="K17" s="3" t="n"/>
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
       <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P17" s="3" t="n"/>
+      <c r="O17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q17" s="3" t="n"/>
-      <c r="R17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S17" s="3" t="n"/>
+      <c r="R17" s="3" t="n"/>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH</t>
+        </is>
+      </c>
       <c r="T17" s="3" t="inlineStr">
         <is>
-          <t>SC; JH</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="U17" s="3" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="V17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W17" s="3" t="n"/>
@@ -1630,12 +1630,12 @@
           <t>An industry that is realised in the processes of facilitating and managing the wagering of money or valuables.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="inlineStr">
@@ -1643,11 +1643,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
+      <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
@@ -1660,15 +1656,15 @@
       </c>
       <c r="P18" s="2" t="n"/>
       <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S18" s="2" t="n"/>
+      <c r="R18" s="2" t="n"/>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>realizable entity</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
@@ -1676,7 +1672,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V18" s="2" t="n"/>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W18" s="2" t="n"/>
     </row>
     <row r="19">
@@ -1695,47 +1695,43 @@
           <t>A governmental organisation set up for a purpose.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">organisation </t>
         </is>
       </c>
-      <c r="F19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>These are set up for purposes such as management of resources, financial oversight of industries, or national security issues. These organizations are typically created by legislative action, but may initially be set up by presidential order as well. The directors of these agencies are typically selected by Presidential appointment</t>
+        </is>
+      </c>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
+      <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
       <c r="M19" s="3" t="n"/>
       <c r="N19" s="3" t="n"/>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P19" s="3" t="inlineStr">
-        <is>
-          <t>These are set up for purposes such as management of resources, financial oversight of industries, or national security issues. These organizations are typically created by legislative action, but may initially be set up by presidential order as well. The directors of these agencies are typically selected by Presidential appointment</t>
-        </is>
-      </c>
+      <c r="O19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n"/>
-      <c r="R19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S19" s="3" t="n"/>
+      <c r="R19" s="3" t="n"/>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="U19" s="3" t="inlineStr">
@@ -1743,7 +1739,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V19" s="3" t="n"/>
+      <c r="V19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W19" s="3" t="n"/>
     </row>
     <row r="20">
@@ -1764,14 +1764,10 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>An organisation that provides products or services that are used for purposes of improving health or reducing ill-health.</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="inlineStr">
@@ -1779,32 +1775,36 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
-      <c r="O20" s="2" t="n">
-        <v>0</v>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>An organisation that provides products or services that are used for purposes of improving health or reducing ill-health.</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="P20" s="2" t="n"/>
       <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="n"/>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V20" s="2" t="n"/>
+      <c r="V20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="W20" s="2" t="n"/>
     </row>
     <row r="21">
@@ -1823,12 +1823,12 @@
           <t>An organisation that provides healthcare.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="inlineStr">
@@ -1836,11 +1836,7 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
@@ -1848,20 +1844,20 @@
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="P21" s="2" t="n"/>
       <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="n"/>
+      <c r="R21" s="2" t="n"/>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
@@ -1869,7 +1865,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V21" s="2" t="n"/>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W21" s="2" t="n"/>
     </row>
     <row r="22">
@@ -1888,51 +1888,51 @@
           <t xml:space="preserve">An e-cigarette company that has no commercial or financial association with a tobacco company. </t>
         </is>
       </c>
-      <c r="D22" s="3" t="n"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>e-cigarette company</t>
+        </is>
+      </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>e-cigarette company</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="n"/>
+          <t xml:space="preserve">Independent vape company; Independent vape business; vape company </t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>(Note: This is intended to include ownership, investment or sharing of resources.)</t>
+        </is>
+      </c>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
+      <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
       <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Independent vape company; Independent vape business; vape company </t>
-        </is>
-      </c>
-      <c r="O22" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="N22" s="3" t="n"/>
+      <c r="O22" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>(Note: This is intended to include ownership, investment or sharing of resources.)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="Q22" s="3" t="n"/>
-      <c r="R22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S22" s="3" t="n"/>
+      <c r="R22" s="3" t="n"/>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="U22" s="3" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="V22" s="3" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W22" s="3" t="n"/>
@@ -1963,47 +1963,47 @@
           <t>A realizable entity that inheres in a collection of organisations, people, equipment and resources and is realised in processes of production, distribution or service provision, and is characterised by a common purpose or set of related economic activities.</t>
         </is>
       </c>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>claude.ai</t>
-        </is>
-      </c>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
+      <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
       <c r="L23" s="4" t="n"/>
       <c r="M23" s="4" t="n"/>
       <c r="N23" s="4" t="n"/>
-      <c r="O23" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P23" s="4" t="n"/>
+      <c r="O23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q23" s="4" t="n"/>
-      <c r="R23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S23" s="4" t="n"/>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>claude.ai</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>JH; SC; RW</t>
+        </is>
+      </c>
       <c r="T23" s="4" t="inlineStr">
         <is>
-          <t>JH; SC; RW</t>
+          <t>realizable entity</t>
         </is>
       </c>
       <c r="U23" s="4" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="V23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W23" s="4" t="n"/>
@@ -2034,12 +2034,12 @@
           <t>A process undertaken by an organisation with the aim of increasing use of a product or service.</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
+      <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
       <c r="H24" s="4" t="inlineStr">
@@ -2047,30 +2047,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
+      <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="n"/>
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
       <c r="N24" s="4" t="n"/>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P24" s="4" t="n"/>
+      <c r="O24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q24" s="4" t="n"/>
-      <c r="R24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T24" s="4" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>process</t>
         </is>
       </c>
       <c r="U24" s="4" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="V24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W24" s="4" t="n"/>
@@ -2101,12 +2101,12 @@
           <t xml:space="preserve">An organisation which is involved in the prevention, diagnosis, treatment and care of people. </t>
         </is>
       </c>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">organisation </t>
         </is>
       </c>
+      <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="inlineStr">
@@ -2114,30 +2114,26 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Role </t>
-        </is>
-      </c>
+      <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
-      <c r="O25" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="O25" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="P25" s="3" t="n"/>
       <c r="Q25" s="3" t="n"/>
-      <c r="R25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S25" s="3" t="n"/>
+      <c r="R25" s="3" t="n"/>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="T25" s="3" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t xml:space="preserve">Role </t>
         </is>
       </c>
       <c r="U25" s="3" t="inlineStr">
@@ -2145,7 +2141,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V25" s="3" t="n"/>
+      <c r="V25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W25" s="3" t="n"/>
     </row>
     <row r="26">
@@ -2164,28 +2164,20 @@
           <t>An organization dedicated to furthering a particular social cause or advocating for a shared point of view. In economic terms, it is an organization that uses its surplus of the revenues to further achieve its ultimate objective, rather than distributing its income to the organization's shareholders, leaders, or members.</t>
         </is>
       </c>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/GSSO_004615</t>
-        </is>
-      </c>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="n"/>
       <c r="L26" s="3" t="n"/>
@@ -2193,20 +2185,24 @@
       <c r="N26" s="3" t="n"/>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="P26" s="3" t="n"/>
       <c r="Q26" s="3" t="n"/>
       <c r="R26" s="3" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="S26" s="3" t="n"/>
+          <t>http://purl.obolibrary.org/obo/GSSO_004615</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U26" s="3" t="inlineStr">
@@ -2214,7 +2210,11 @@
           <t>Pre-proposed</t>
         </is>
       </c>
-      <c r="V26" s="3" t="n"/>
+      <c r="V26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W26" s="3" t="n"/>
     </row>
     <row r="27">
@@ -2233,52 +2233,52 @@
           <t>A material entity which can play roles, has members, and has a set of organization rules. Members of organizations are either organizations themselves or individual people. Members can bear specific organization member roles that are determined in the organization rules. The organization rules also determine how decisions are made on behalf of the organization by the organization members.</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>The definition from OBI has been slightly changed to refer to 'material entity' rather than 'continuant entity'</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>1</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>OBI:0000245</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>OBI:0000245</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>The definition from OBI has been slightly changed to refer to 'material entity' rather than 'continuant entity'</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
         <is>
           <t>false</t>
-        </is>
-      </c>
-      <c r="R27" t="n">
-        <v>1</v>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>External</t>
         </is>
       </c>
     </row>
@@ -2298,12 +2298,12 @@
           <t>An aggregate of organisations.</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
+      <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
       <c r="H28" s="5" t="inlineStr">
@@ -2324,23 +2324,23 @@
       </c>
       <c r="P28" s="5" t="n"/>
       <c r="Q28" s="5" t="n"/>
-      <c r="R28" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="S28" s="5" t="n"/>
-      <c r="T28" s="5" t="inlineStr">
+      <c r="R28" s="5" t="n"/>
+      <c r="S28" s="5" t="inlineStr">
         <is>
           <t>JH; RW</t>
         </is>
       </c>
+      <c r="T28" s="5" t="n"/>
       <c r="U28" s="5" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="V28" s="5" t="n"/>
+      <c r="V28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W28" s="5" t="n"/>
     </row>
     <row r="29">
@@ -2361,14 +2361,10 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>A commercial organisation that deals with pharmaceutical products or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
           <t>commercial organisation</t>
         </is>
       </c>
+      <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="inlineStr">
@@ -2376,32 +2372,36 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="n"/>
-      <c r="N29" s="2" t="n"/>
-      <c r="O29" s="2" t="n">
-        <v>0</v>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>A commercial organisation that deals with pharmaceutical products or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="P29" s="2" t="n"/>
       <c r="Q29" s="2" t="n"/>
-      <c r="R29" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="R29" s="2" t="n"/>
       <c r="S29" s="2" t="n"/>
-      <c r="T29" s="2" t="n"/>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V29" s="2" t="n"/>
+      <c r="V29" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="W29" s="2" t="n"/>
     </row>
     <row r="30">
@@ -2422,14 +2422,10 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>An organisation that makes or provides products or services that people use for enjoyment, entertainment, or leisure activities.</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="inlineStr">
@@ -2437,32 +2433,36 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I30" s="2" t="n"/>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="n"/>
-      <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="n">
-        <v>0</v>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>An organisation that makes or provides products or services that people use for enjoyment, entertainment, or leisure activities.</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="n"/>
-      <c r="R30" s="2" t="b">
-        <v>1</v>
-      </c>
+      <c r="R30" s="2" t="n"/>
       <c r="S30" s="2" t="n"/>
-      <c r="T30" s="2" t="n"/>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
       <c r="U30" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V30" s="2" t="n"/>
+      <c r="V30" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="W30" s="2" t="n"/>
     </row>
     <row r="31">
@@ -2481,47 +2481,43 @@
           <t>An organization that has responsibility over or for the legislation (acts and regulations) for a given sector of the government.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/OBI_0000450</t>
-        </is>
-      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
       <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I31" s="2" t="n"/>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="O31" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="P31" s="2" t="n"/>
       <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S31" s="2" t="n"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/OBI_0000450</t>
+        </is>
+      </c>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>SC; RW</t>
+        </is>
+      </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>SC; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U31" s="2" t="inlineStr">
@@ -2529,7 +2525,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V31" s="2" t="n"/>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W31" s="2" t="n"/>
     </row>
     <row r="32">
@@ -2548,10 +2548,14 @@
           <t>An organization that provides funding for research.</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>organisation</t>
+        </is>
+      </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>organisation</t>
+          <t>funder</t>
         </is>
       </c>
       <c r="F32" s="2" t="n"/>
@@ -2561,34 +2565,26 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="n"/>
       <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>funder</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S32" s="2" t="n"/>
+      <c r="R32" s="2" t="n"/>
+      <c r="S32" s="2" t="inlineStr">
+        <is>
+          <t>SC; KS; RW</t>
+        </is>
+      </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>SC; KS; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr">
@@ -2596,7 +2592,11 @@
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V32" s="2" t="n"/>
+      <c r="V32" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="W32" s="2" t="n"/>
     </row>
     <row r="33">
@@ -2615,47 +2615,47 @@
           <t>An organisation formed with a goal to have its members conduct investigations.</t>
         </is>
       </c>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">organisation </t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>http://purl.obolibrary.org/obo/OBI_0000828</t>
-        </is>
-      </c>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="n"/>
       <c r="L33" s="3" t="n"/>
       <c r="M33" s="3" t="n"/>
       <c r="N33" s="3" t="n"/>
-      <c r="O33" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P33" s="3" t="n"/>
+      <c r="O33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>RW; CN</t>
+        </is>
+      </c>
       <c r="Q33" s="3" t="n"/>
-      <c r="R33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S33" s="3" t="n"/>
+      <c r="R33" s="3" t="inlineStr">
+        <is>
+          <t>http://purl.obolibrary.org/obo/OBI_0000828</t>
+        </is>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T33" s="3" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U33" s="3" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="V33" s="3" t="inlineStr">
         <is>
-          <t>RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W33" s="3" t="n"/>
@@ -2686,12 +2686,12 @@
           <t>An organisation that sells some product directly to users of that product.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
+      <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="inlineStr">
@@ -2699,118 +2699,118 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I34" s="2" t="n"/>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P34" s="2" t="n"/>
+      <c r="O34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="n">
+      <c r="R34" s="2" t="n"/>
+      <c r="S34" s="2" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="V34" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>ADDICTO:0000435</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>tobacco company</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>A commercial organisation that is engaged in the growth, manufacture, preparation for sale, shipment, advertisement, or distribution of tobacco, or a tobacco-containing product, or is at least partly owned by such an organisation.</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>organisation</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n"/>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>This excludes law firms acting for the TI. It also excludes organisations that are solely NRT manufacturers and e-cig manufacturers even though nicotine is derived from tobacco.</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="n"/>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>A commercial organisation that deals with tobacco in any part of the process from growing it to getting it to consumers, or is at least partly owned by such an organisation.</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="S34" s="2" t="n"/>
-      <c r="T34" s="2" t="inlineStr">
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="n"/>
+      <c r="R35" s="4" t="n"/>
+      <c r="S35" s="4" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="U34" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="V34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> RW; CN</t>
-        </is>
-      </c>
-      <c r="W34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>ADDICTO:0000435</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>tobacco company</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>A commercial organisation that is engaged in the growth, manufacture, preparation for sale, shipment, advertisement, or distribution of tobacco, or a tobacco-containing product, or is at least partly owned by such an organisation.</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>A commercial organisation that deals with tobacco in any part of the process from growing it to getting it to consumers, or is at least partly owned by such an organisation.</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>organisation</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="T35" s="4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
-      <c r="L35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="N35" s="3" t="n"/>
-      <c r="O35" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P35" s="3" t="inlineStr">
-        <is>
-          <t>This excludes law firms acting for the TI. It also excludes NRT manufacturers and e-cig manufacturers even though nicotine is derived from tobacco.</t>
-        </is>
-      </c>
-      <c r="Q35" s="3" t="n"/>
-      <c r="R35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S35" s="3" t="n"/>
-      <c r="T35" s="3" t="inlineStr">
-        <is>
-          <t>SC; JH; RW</t>
-        </is>
-      </c>
-      <c r="U35" s="3" t="inlineStr">
-        <is>
-          <t>Pre-proposed</t>
-        </is>
-      </c>
-      <c r="V35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> RW; CN</t>
-        </is>
-      </c>
-      <c r="W35" s="3" t="n"/>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>Discussed</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2828,12 +2828,12 @@
           <t>An industry that is realised in the manufacture or sale of tobacco and tobacco-containing products.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
+      <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="inlineStr">
@@ -2841,30 +2841,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>realizable entity</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="n"/>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
       <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="n"/>
+      <c r="O36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q36" s="2" t="n"/>
-      <c r="R36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S36" s="2" t="n"/>
+      <c r="R36" s="2" t="n"/>
+      <c r="S36" s="2" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>realizable entity</t>
         </is>
       </c>
       <c r="U36" s="2" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="V36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W36" s="2" t="n"/>
@@ -2895,12 +2895,12 @@
           <t>A facility that retails tobacco.</t>
         </is>
       </c>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>facility</t>
         </is>
       </c>
+      <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="inlineStr">
@@ -2908,30 +2908,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="3" t="n"/>
       <c r="L37" s="3" t="n"/>
       <c r="M37" s="3" t="n"/>
       <c r="N37" s="3" t="n"/>
-      <c r="O37" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P37" s="3" t="n"/>
+      <c r="O37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q37" s="3" t="n"/>
-      <c r="R37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S37" s="3" t="n"/>
+      <c r="R37" s="3" t="n"/>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U37" s="3" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="V37" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W37" s="3" t="n"/>
@@ -2962,12 +2962,12 @@
           <t xml:space="preserve">A retailer that sells tobacco products. </t>
         </is>
       </c>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>retailer</t>
         </is>
       </c>
+      <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="inlineStr">
@@ -2975,30 +2975,30 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="n"/>
       <c r="L38" s="3" t="n"/>
       <c r="M38" s="3" t="n"/>
       <c r="N38" s="3" t="n"/>
-      <c r="O38" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P38" s="3" t="n"/>
+      <c r="O38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q38" s="3" t="n"/>
-      <c r="R38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="S38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>SC; JH; RW</t>
+        </is>
+      </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>SC; JH; RW</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U38" s="3" t="inlineStr">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="V38" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W38" s="3" t="n"/>
@@ -3031,14 +3031,10 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>A commercial organisation that deals with vaping devices or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
           <t>commercial organisation</t>
         </is>
       </c>
+      <c r="E39" s="2" t="n"/>
       <c r="F39" s="2" t="n"/>
       <c r="G39" s="2" t="n"/>
       <c r="H39" s="2" t="inlineStr">
@@ -3046,30 +3042,34 @@
           <t>Organisation</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>material entity</t>
-        </is>
-      </c>
+      <c r="I39" s="2" t="n"/>
       <c r="J39" s="2" t="n"/>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="n"/>
       <c r="M39" s="2" t="n"/>
-      <c r="N39" s="2" t="n"/>
-      <c r="O39" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P39" s="2" t="n"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>A commercial organisation that deals with vaping devices or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> RW; CN</t>
+        </is>
+      </c>
       <c r="Q39" s="2" t="n"/>
-      <c r="R39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S39" s="2" t="n"/>
+      <c r="R39" s="2" t="n"/>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>SC; JH</t>
+        </is>
+      </c>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>SC; JH</t>
+          <t>material entity</t>
         </is>
       </c>
       <c r="U39" s="2" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="V39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RW; CN</t>
+          <t>0</t>
         </is>
       </c>
       <c r="W39" s="2" t="n"/>

</xml_diff>

<commit_message>
Update 7 terms in AddictO_Organisation_Defs.xlsx
</commit_message>
<xml_diff>
--- a/inputs/AddictO_Organisation_Defs.xlsx
+++ b/inputs/AddictO_Organisation_Defs.xlsx
@@ -39,7 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
+        <fgColor rgb="00ffe4b5"/>
       </patternFill>
     </fill>
     <fill>
@@ -49,7 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ffe4b5"/>
+        <fgColor rgb="00ffffff"/>
       </patternFill>
     </fill>
     <fill>
@@ -615,7 +615,7 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V2" s="2" t="n">
@@ -693,69 +693,69 @@
       <c r="W3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ADDICTO:0000411</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>alcohol industry</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>An industry that is realised in the manufacture and sale of alcoholic beverages.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="n"/>
-      <c r="S4" s="4" t="inlineStr">
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>SC; RW</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="U4" s="4" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="n"/>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -955,69 +955,69 @@
       <c r="W7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0000415</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">cannabis industry </t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>An industry that is realised in the manufacture and sale of cannabis.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>SC; RW</t>
         </is>
       </c>
-      <c r="T8" s="2" t="inlineStr">
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="U8" s="2" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="n"/>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1150,71 +1150,71 @@
       <c r="W10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0001101</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">charity </t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">An organisation that raises and distributes funds for charitable purposes. </t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
-      <c r="O11" s="2" t="n">
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="n"/>
+      <c r="O11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="P11" s="4" t="inlineStr">
         <is>
           <t>RW; CN</t>
         </is>
       </c>
-      <c r="Q11" s="2" t="n"/>
-      <c r="R11" s="2" t="n"/>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="Q11" s="4" t="n"/>
+      <c r="R11" s="4" t="n"/>
+      <c r="S11" s="4" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="T11" s="2" t="inlineStr">
+      <c r="T11" s="4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="U11" s="2" t="inlineStr">
+      <c r="U11" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W11" s="2" t="n"/>
+      <c r="V11" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="U12" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V12" s="2" t="n">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V13" s="2" t="n">
@@ -1339,75 +1339,75 @@
       <c r="W13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>ADDICTO:0000420</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>e-cigarette industry</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>An industry that is realised in the manufacture and sale of e-cigarettes, e-cigarette components and e-liquid.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>E-Cig industry</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">I have added here promotion of - this sets industry apart from manufactureres of but also includes these types of company. </t>
         </is>
       </c>
-      <c r="N14" s="4" t="n"/>
-      <c r="O14" s="4" t="n">
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P14" s="4" t="n"/>
-      <c r="Q14" s="4" t="n"/>
-      <c r="R14" s="4" t="n"/>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2" t="inlineStr">
         <is>
           <t>SC; RW</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="T14" s="2" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr">
+      <c r="U14" s="2" t="inlineStr">
         <is>
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V14" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W14" s="4" t="n"/>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1615,69 +1615,69 @@
       <c r="W17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0000424</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>gambling industry</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>An industry that is realised in the processes of facilitating and managing the wagering of money or valuables.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="n"/>
-      <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="n"/>
-      <c r="S18" s="2" t="inlineStr">
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
+      <c r="L18" s="4" t="n"/>
+      <c r="M18" s="4" t="n"/>
+      <c r="N18" s="4" t="n"/>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="n"/>
+      <c r="Q18" s="4" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="inlineStr">
         <is>
           <t>SC; RW</t>
         </is>
       </c>
-      <c r="T18" s="2" t="inlineStr">
+      <c r="T18" s="4" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="U18" s="2" t="inlineStr">
+      <c r="U18" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V18" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W18" s="2" t="n"/>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1754,12 +1754,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>health-improvement organisation</t>
+          <t>health-improvement provider</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>An organisation that has as a function the production, distribution, or provision of goods or services intended to improve health or reduce ill-health.</t>
+          <t>An organisation that is engaged in the production, distribution, or provision of goods or services intended to improve health or reduce ill-health.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V20" s="2" t="n">
@@ -1808,69 +1808,69 @@
       <c r="W20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0001359</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">healthcare organisation </t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>An organisation that provides healthcare.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="n"/>
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="P21" s="2" t="n"/>
-      <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="n"/>
-      <c r="S21" s="2" t="inlineStr">
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="n"/>
+      <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="T21" s="2" t="inlineStr">
+      <c r="T21" s="4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="U21" s="2" t="inlineStr">
+      <c r="U21" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V21" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W21" s="2" t="n"/>
+      <c r="V21" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1948,142 +1948,142 @@
       <c r="W22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>ADDICTO:0000428</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>A realizable entity that inheres in a collection of organisations, people, equipment and resources and is realised in processes of production, distribution or service provision, and is characterised by a common purpose or set of related economic activities.</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="n"/>
-      <c r="J23" s="4" t="n"/>
-      <c r="K23" s="4" t="n"/>
-      <c r="L23" s="4" t="n"/>
-      <c r="M23" s="4" t="n"/>
-      <c r="N23" s="4" t="n"/>
-      <c r="O23" s="4" t="n">
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="n"/>
+      <c r="O23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> RW; CN</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="n"/>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" s="2" t="inlineStr">
         <is>
           <t>claude.ai</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr">
+      <c r="S23" s="2" t="inlineStr">
         <is>
           <t>JH; SC; RW</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
+      <c r="T23" s="2" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
+      <c r="U23" s="2" t="inlineStr">
         <is>
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V23" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W23" s="4" t="n"/>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>ADDICTO:0000429</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>marketing</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>A process undertaken by an organisation with the aim of increasing use of a product or service.</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="n"/>
-      <c r="J24" s="4" t="n"/>
-      <c r="K24" s="4" t="n"/>
-      <c r="L24" s="4" t="n"/>
-      <c r="M24" s="4" t="n"/>
-      <c r="N24" s="4" t="n"/>
-      <c r="O24" s="4" t="n">
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P24" s="4" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> RW; CN</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="n"/>
-      <c r="R24" s="4" t="n"/>
-      <c r="S24" s="4" t="inlineStr">
+      <c r="Q24" s="2" t="n"/>
+      <c r="R24" s="2" t="n"/>
+      <c r="S24" s="2" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
+      <c r="T24" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr">
+      <c r="U24" s="2" t="inlineStr">
         <is>
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V24" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W24" s="4" t="n"/>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A commercial organisation that is engaged in the manufacture, preparation for sale, shipment, advertisement, or distribution of  a pharmaceutical product or part of such a product, or is at least partly owned by such an organisation.</t>
+          <t>A commercial organisation that is engaged in the manufacture, preparation for sale, shipment, advertisement, or distribution of  a pharmaceutical product, or is at least partly owned by such an organisation.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2379,7 +2379,7 @@
       <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>A commercial organisation that deals with pharmaceutical products or their parts in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
+          <t>A commercial organisation that deals with pharmaceutical products in any part of the process from manufacturing them to getting them to consumers, or is at least partly owned by such an organisation.</t>
         </is>
       </c>
       <c r="O29" s="2" t="b">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V29" s="2" t="n">
@@ -2412,12 +2412,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>recreational organisation</t>
+          <t>recreational consumer product organisation</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>An organisation that has as a function the production, distribution, or provision of goods or services intended for recreational use by consumers.</t>
+          <t>An organisation that is engaged in the production, distribution, or provision of goods or services intended for recreational use by consumers.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2440,7 +2440,7 @@
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>An organisation that makes or provides products or services that people use for enjoyment, entertainment, or leisure activities.</t>
+          <t>An organisation that makes or provides consumer products or services that people use for enjoyment, entertainment, or leisure activities.</t>
         </is>
       </c>
       <c r="O30" s="2" t="b">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="U30" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V30" s="2" t="n">
@@ -2466,138 +2466,138 @@
       <c r="W30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0001102</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">regulatory agency </t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>An organization that has responsibility over or for the legislation (acts and regulations) for a given sector of the government.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
-      <c r="N31" s="2" t="n"/>
-      <c r="O31" s="2" t="n">
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="4" t="n"/>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4" t="n"/>
+      <c r="O31" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="inlineStr">
+      <c r="P31" s="4" t="n"/>
+      <c r="Q31" s="4" t="n"/>
+      <c r="R31" s="4" t="inlineStr">
         <is>
           <t>http://purl.obolibrary.org/obo/OBI_0000450</t>
         </is>
       </c>
-      <c r="S31" s="2" t="inlineStr">
+      <c r="S31" s="4" t="inlineStr">
         <is>
           <t>SC; RW</t>
         </is>
       </c>
-      <c r="T31" s="2" t="inlineStr">
+      <c r="T31" s="4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="U31" s="2" t="inlineStr">
+      <c r="U31" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V31" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W31" s="2" t="n"/>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0000880</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">research grant awarding body </t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>An organization that provides funding for research.</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>funder</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="n"/>
-      <c r="N32" s="2" t="n"/>
-      <c r="O32" s="2" t="n">
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="n"/>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="4" t="n"/>
+      <c r="M32" s="4" t="n"/>
+      <c r="N32" s="4" t="n"/>
+      <c r="O32" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="n"/>
-      <c r="S32" s="2" t="inlineStr">
+      <c r="P32" s="4" t="n"/>
+      <c r="Q32" s="4" t="n"/>
+      <c r="R32" s="4" t="n"/>
+      <c r="S32" s="4" t="inlineStr">
         <is>
           <t>SC; KS; RW</t>
         </is>
       </c>
-      <c r="T32" s="2" t="inlineStr">
+      <c r="T32" s="4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="U32" s="2" t="inlineStr">
+      <c r="U32" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V32" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W32" s="2" t="n"/>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2671,213 +2671,213 @@
       <c r="W33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0000433</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>retailer</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>An organisation that sells some product directly to users of that product.</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
-      <c r="N34" s="2" t="n"/>
-      <c r="O34" s="2" t="n">
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="n"/>
+      <c r="J34" s="4" t="n"/>
+      <c r="K34" s="4" t="n"/>
+      <c r="L34" s="4" t="n"/>
+      <c r="M34" s="4" t="n"/>
+      <c r="N34" s="4" t="n"/>
+      <c r="O34" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P34" s="2" t="inlineStr">
+      <c r="P34" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> RW; CN</t>
         </is>
       </c>
-      <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="n"/>
-      <c r="S34" s="2" t="inlineStr">
+      <c r="Q34" s="4" t="n"/>
+      <c r="R34" s="4" t="n"/>
+      <c r="S34" s="4" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="T34" s="2" t="inlineStr">
+      <c r="T34" s="4" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="U34" s="2" t="inlineStr">
+      <c r="U34" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V34" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W34" s="2" t="n"/>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>ADDICTO:0000435</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>tobacco company</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>A commercial organisation that is engaged in the growth, manufacture, preparation for sale, shipment, advertisement, or distribution of tobacco, or a tobacco-containing product, or is at least partly owned by such an organisation.</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>organisation</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n"/>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>This excludes law firms acting for the TI. It also excludes organisations that are solely NRT manufacturers and e-cig manufacturers even though nicotine is derived from tobacco.</t>
         </is>
       </c>
-      <c r="G35" s="4" t="n"/>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
-      <c r="L35" s="4" t="n"/>
-      <c r="M35" s="4" t="n"/>
-      <c r="N35" s="4" t="inlineStr">
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>A commercial organisation that deals with tobacco in any part of the process from growing it to getting it to consumers, or is at least partly owned by such an organisation.</t>
         </is>
       </c>
-      <c r="O35" s="4" t="n">
+      <c r="O35" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P35" s="4" t="inlineStr">
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> RW; CN</t>
         </is>
       </c>
-      <c r="Q35" s="4" t="n"/>
-      <c r="R35" s="4" t="n"/>
-      <c r="S35" s="4" t="inlineStr">
+      <c r="Q35" s="2" t="n"/>
+      <c r="R35" s="2" t="n"/>
+      <c r="S35" s="2" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="T35" s="4" t="inlineStr">
+      <c r="T35" s="2" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="U35" s="4" t="inlineStr">
+      <c r="U35" s="2" t="inlineStr">
         <is>
           <t>Discussed</t>
         </is>
       </c>
-      <c r="V35" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W35" s="4" t="n"/>
+      <c r="V35" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>ADDICTO:0000436</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>tobacco industry</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>An industry that is realised in the manufacture or sale of tobacco and tobacco-containing products.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n">
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Organisation</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="n"/>
+      <c r="O36" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="P36" s="2" t="inlineStr">
+      <c r="P36" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> RW; CN</t>
         </is>
       </c>
-      <c r="Q36" s="2" t="n"/>
-      <c r="R36" s="2" t="n"/>
-      <c r="S36" s="2" t="inlineStr">
+      <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="inlineStr">
         <is>
           <t>SC; JH; RW</t>
         </is>
       </c>
-      <c r="T36" s="2" t="inlineStr">
+      <c r="T36" s="4" t="inlineStr">
         <is>
           <t>realizable entity</t>
         </is>
       </c>
-      <c r="U36" s="2" t="inlineStr">
+      <c r="U36" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="V36" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="W36" s="2" t="n"/>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Discussed</t>
         </is>
       </c>
       <c r="V39" s="2" t="inlineStr">

</xml_diff>